<commit_message>
Pre Market Thu 2026-07-09
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-07-09.xlsx
+++ b/market-prep/Pre Market 2026-07-09.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7478,64</t>
+          <t>7482,71</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29195,39</t>
+          <t>29252,56</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2956,37</t>
+          <t>2956,39</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52336,81</t>
+          <t>52348,39</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6++</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4076,21</t>
+          <t>4074,43</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>58,32</t>
+          <t>58,30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1586,70</t>
+          <t>1582,70</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>78,54</t>
+          <t>78,02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>62171,08</t>
+          <t>62020,40</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1735,98</t>
+          <t>1732,77</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3,91%</t>
+          <t>4,77%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7480,38</t>
+          <t>7482,71</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>